<commit_message>
docs: Populate version control matrix with complete history of 9 Bolts and Intent IDs
</commit_message>
<xml_diff>
--- a/docs/Matriz de registro(MODELO DE CONTROL DE VERSIONES).xlsx
+++ b/docs/Matriz de registro(MODELO DE CONTROL DE VERSIONES).xlsx
@@ -1823,15 +1823,19 @@
       <c r="BY4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="99" t="n"/>
+      <c r="A5" s="99" t="inlineStr">
+        <is>
+          <t>I001</t>
+        </is>
+      </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>BOLT-VT-001</t>
+          <t>BOLT-VT-000</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Refactorizacion de Codigo Limpio y Cobertura de Pruebas en SonarQube</t>
+          <t>Configuracion e inicializacion del esquema de base de datos relacional y arquitectura base de FastAPI.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -1841,17 +1845,17 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Seguridad y Calidad de Codigo</t>
+          <t>Base de Datos e Infraestructura</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>HU-001</t>
+          <t>HU-000</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
@@ -1866,7 +1870,7 @@
       </c>
       <c r="J5" s="53" t="inlineStr">
         <is>
-          <t>Se identifico la necesidad de resolver la complejidad cognitiva en la inferencia YOLO.</t>
+          <t>Se definio la estructura base para el almacenamiento persistente de infracciones.</t>
         </is>
       </c>
       <c r="K5" s="1" t="inlineStr">
@@ -1876,7 +1880,7 @@
       </c>
       <c r="L5" s="1" t="inlineStr">
         <is>
-          <t>plan_de_implementacion.md anterior</t>
+          <t>Requerimiento de almacenamiento de datos de vehiculos y conductores.</t>
         </is>
       </c>
       <c r="M5" s="1" t="inlineStr">
@@ -1886,7 +1890,7 @@
       </c>
       <c r="N5" s="1" t="inlineStr">
         <is>
-          <t>ia_service.py y yolo_predictor.py</t>
+          <t>Separacion de tablas para evitar redundancias de datos.</t>
         </is>
       </c>
       <c r="O5" s="1" t="n"/>
@@ -1897,7 +1901,7 @@
       </c>
       <c r="Q5" s="1" t="inlineStr">
         <is>
-          <t>plan_de_implementacion.md</t>
+          <t>Modelo entidad-relacion de 20 tablas documentado.</t>
         </is>
       </c>
       <c r="R5" s="1" t="inlineStr">
@@ -1907,7 +1911,7 @@
       </c>
       <c r="S5" s="53" t="inlineStr">
         <is>
-          <t>Commit 8ba35f6</t>
+          <t>Commit a87436a</t>
         </is>
       </c>
       <c r="T5" s="1" t="inlineStr">
@@ -1917,7 +1921,7 @@
       </c>
       <c r="U5" s="1" t="inlineStr">
         <is>
-          <t>Pytest suite passed (34 tests)</t>
+          <t>Pruebas de conexion local aprobadas.</t>
         </is>
       </c>
       <c r="V5" s="1" t="n"/>
@@ -1928,7 +1932,7 @@
       </c>
       <c r="X5" s="1" t="inlineStr">
         <is>
-          <t>Despliegue en Render</t>
+          <t>Despliegue local inicial de base de datos.</t>
         </is>
       </c>
       <c r="Y5" s="29" t="n"/>
@@ -1940,7 +1944,7 @@
       </c>
       <c r="AB5" s="1" t="inlineStr">
         <is>
-          <t>backend/app/services</t>
+          <t>Esquema guardado en docs/database_schema.sql.</t>
         </is>
       </c>
       <c r="AC5" s="38" t="inlineStr">
@@ -1950,7 +1954,7 @@
       </c>
       <c r="AD5" s="1" t="inlineStr">
         <is>
-          <t>ia_service.py y yolo_predictor.py</t>
+          <t>Aislamiento de la logica de datos en el script SQL.</t>
         </is>
       </c>
       <c r="AE5" s="1" t="inlineStr">
@@ -1960,7 +1964,7 @@
       </c>
       <c r="AF5" s="1" t="inlineStr">
         <is>
-          <t>Estructura limpia sin duplicados</t>
+          <t>Diseno normalizado en tercera forma normal (3FN).</t>
         </is>
       </c>
       <c r="AG5" s="1" t="inlineStr">
@@ -1970,7 +1974,7 @@
       </c>
       <c r="AH5" s="1" t="inlineStr">
         <is>
-          <t>Modularizacion de reglas de transito y YOLO</t>
+          <t>Separacion fisica de almacenamiento y logica del backend.</t>
         </is>
       </c>
       <c r="AI5" s="1" t="n"/>
@@ -1981,7 +1985,7 @@
       </c>
       <c r="AK5" s="1" t="inlineStr">
         <is>
-          <t>PEP 8</t>
+          <t>Uso de minusculas y snake_case para nombres de tablas y columnas.</t>
         </is>
       </c>
       <c r="AL5" s="1" t="inlineStr">
@@ -1991,7 +1995,7 @@
       </c>
       <c r="AM5" s="1" t="inlineStr">
         <is>
-          <t>Modulos y nombres estandar</t>
+          <t>Estructura estandar de base de datos SQL.</t>
         </is>
       </c>
       <c r="AN5" s="1" t="inlineStr">
@@ -2001,7 +2005,7 @@
       </c>
       <c r="AO5" t="inlineStr">
         <is>
-          <t>Sin dependencias extras</t>
+          <t>Sin librerias adicionales para definicion SQL.</t>
         </is>
       </c>
       <c r="AP5" s="1" t="n"/>
@@ -2013,7 +2017,7 @@
       </c>
       <c r="AS5" s="1" t="inlineStr">
         <is>
-          <t>BOLT-VT-001</t>
+          <t>BOLT-VT-000</t>
         </is>
       </c>
       <c r="AT5" s="1" t="inlineStr">
@@ -2023,7 +2027,7 @@
       </c>
       <c r="AU5" s="1" t="inlineStr">
         <is>
-          <t>plan_de_implementacion.md</t>
+          <t>HU-000</t>
         </is>
       </c>
       <c r="AV5" s="1" t="inlineStr">
@@ -2033,7 +2037,7 @@
       </c>
       <c r="AW5" s="1" t="inlineStr">
         <is>
-          <t>Commit 8ba35f6</t>
+          <t>Commit a87436a</t>
         </is>
       </c>
       <c r="AX5" s="1" t="inlineStr">
@@ -2053,7 +2057,7 @@
       </c>
       <c r="BA5" s="1" t="inlineStr">
         <is>
-          <t>Render build success logs</t>
+          <t>Base de datos cargada localmente.</t>
         </is>
       </c>
       <c r="BB5" s="1" t="n"/>
@@ -2065,7 +2069,7 @@
       </c>
       <c r="BE5" s="1" t="inlineStr">
         <is>
-          <t>Validacion local exitosa</t>
+          <t>Verificacion de relaciones y claves foraneas.</t>
         </is>
       </c>
       <c r="BF5" s="1" t="inlineStr">
@@ -2075,7 +2079,7 @@
       </c>
       <c r="BG5" s="1" t="inlineStr">
         <is>
-          <t>Analisis YOLO modular</t>
+          <t>Creacion exitosa de las 20 tablas relacionales.</t>
         </is>
       </c>
       <c r="BH5" s="1" t="inlineStr">
@@ -2085,7 +2089,7 @@
       </c>
       <c r="BI5" s="1" t="inlineStr">
         <is>
-          <t>Reglas heuristicas funcionando</t>
+          <t>No afecta otras configuraciones del sistema.</t>
         </is>
       </c>
       <c r="BJ5" s="1" t="inlineStr">
@@ -2095,7 +2099,7 @@
       </c>
       <c r="BK5" s="1" t="inlineStr">
         <is>
-          <t>Cero bugs reportados en QA</t>
+          <t>Migracion inicial libre de errores.</t>
         </is>
       </c>
       <c r="BL5" s="1" t="n"/>
@@ -2106,7 +2110,7 @@
       </c>
       <c r="BN5" s="1" t="inlineStr">
         <is>
-          <t>SonarQube Quality Gate Passed (0 violations)</t>
+          <t>Esquema SQL verificado sin advertencias de sintaxis.</t>
         </is>
       </c>
       <c r="BO5" s="1" t="inlineStr">
@@ -2116,7 +2120,7 @@
       </c>
       <c r="BP5" s="1" t="inlineStr">
         <is>
-          <t>Sin vulnerabilidades reportadas</t>
+          <t>Restriccion de acceso mediante variables de entorno.</t>
         </is>
       </c>
       <c r="BQ5" s="1" t="inlineStr">
@@ -2126,7 +2130,7 @@
       </c>
       <c r="BR5" s="1" t="inlineStr">
         <is>
-          <t>Pytest al 100% de cobertura</t>
+          <t>Script SQL ejecutado con exito.</t>
         </is>
       </c>
       <c r="BS5" s="1" t="inlineStr">
@@ -2136,7 +2140,7 @@
       </c>
       <c r="BT5" s="53" t="inlineStr">
         <is>
-          <t>walkthrough.md aprobado por usuario</t>
+          <t>Aprobacion de arquitectura por el equipo.</t>
         </is>
       </c>
       <c r="BU5" s="1" t="n"/>
@@ -2148,12 +2152,12 @@
       </c>
       <c r="BX5" s="9" t="inlineStr">
         <is>
-          <t>Refactorizacion integral del backend para solucionar complejidad cognitiva y duplicados de SonarQube.</t>
+          <t>Configuracion base de base de datos de 20 tablas establecida para la gestion del sistema de infracciones.</t>
         </is>
       </c>
       <c r="BY5" s="1" t="inlineStr">
         <is>
-          <t>La cobertura del backend es del 100% en codigo nuevo.</t>
+          <t>Migrar a PostgreSQL en entorno productivo mediante variables de entorno en Render.</t>
         </is>
       </c>
     </row>
@@ -2161,32 +2165,32 @@
       <c r="A6" s="115" t="n"/>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>BOLT-VT-002</t>
+          <t>BOLT-VT-001</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>Alineacion de bounding boxes y asociacion de placa semilla</t>
+          <t>Configuracion de archivos de despliegue render.yaml y setup de CORS frontend/backend.</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>YOLOv8 + EasyOCR</t>
+          <t>Gemini Code Assist</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>Gestion de Infracciones de Transito</t>
+          <t>Despliegue y Hosting</t>
         </is>
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>HU-002</t>
+          <t>HU-001</t>
         </is>
       </c>
       <c r="H6" s="9" t="inlineStr">
@@ -2201,7 +2205,7 @@
       </c>
       <c r="J6" s="53" t="inlineStr">
         <is>
-          <t>Se detecto la desalineacion de la caja del semaforo en la copa del arbol.</t>
+          <t>Requerimiento para desplegar la app en la nube de Render de forma automatizada.</t>
         </is>
       </c>
       <c r="K6" s="1" t="inlineStr">
@@ -2211,7 +2215,7 @@
       </c>
       <c r="L6" s="1" t="inlineStr">
         <is>
-          <t>plan de implementacion</t>
+          <t>Configuracion de infraestructura de hosting.</t>
         </is>
       </c>
       <c r="M6" s="1" t="inlineStr">
@@ -2221,7 +2225,7 @@
       </c>
       <c r="N6" s="1" t="inlineStr">
         <is>
-          <t>yolo_predictor.py y rules.py</t>
+          <t>Creacion de archivo render.yaml en la raiz del proyecto.</t>
         </is>
       </c>
       <c r="O6" s="1" t="n"/>
@@ -2232,7 +2236,7 @@
       </c>
       <c r="Q6" s="1" t="inlineStr">
         <is>
-          <t>plan de implementacion</t>
+          <t>Arquitectura de despliegue distribuida en Render.</t>
         </is>
       </c>
       <c r="R6" s="1" t="inlineStr">
@@ -2242,7 +2246,7 @@
       </c>
       <c r="S6" s="53" t="inlineStr">
         <is>
-          <t>Commit 8754814</t>
+          <t>Commit 63a14b0</t>
         </is>
       </c>
       <c r="T6" s="1" t="inlineStr">
@@ -2252,7 +2256,7 @@
       </c>
       <c r="U6" s="1" t="inlineStr">
         <is>
-          <t>Pytest suite passed (34 tests)</t>
+          <t>Linter de yaml superado.</t>
         </is>
       </c>
       <c r="V6" s="1" t="n"/>
@@ -2263,7 +2267,7 @@
       </c>
       <c r="X6" s="1" t="inlineStr">
         <is>
-          <t>Despliegue en Render</t>
+          <t>Blueprint de Render desplegado.</t>
         </is>
       </c>
       <c r="Y6" s="29" t="n"/>
@@ -2275,7 +2279,7 @@
       </c>
       <c r="AB6" s="1" t="inlineStr">
         <is>
-          <t>backend/app/services</t>
+          <t>Ubicacion de render.yaml en la raiz.</t>
         </is>
       </c>
       <c r="AC6" s="38" t="inlineStr">
@@ -2285,7 +2289,7 @@
       </c>
       <c r="AD6" s="1" t="inlineStr">
         <is>
-          <t>yolo_predictor.py y rules.py</t>
+          <t>CORS configurado dinamicamente en backend/app/main.py.</t>
         </is>
       </c>
       <c r="AE6" s="1" t="inlineStr">
@@ -2295,7 +2299,7 @@
       </c>
       <c r="AF6" s="1" t="inlineStr">
         <is>
-          <t>Sin redundancias de archivos</t>
+          <t>Evita duplicacion de archivos de infraestructura.</t>
         </is>
       </c>
       <c r="AG6" s="1" t="inlineStr">
@@ -2305,7 +2309,7 @@
       </c>
       <c r="AH6" s="1" t="inlineStr">
         <is>
-          <t>Deteccion e inferencia en predictor, validacion en rules</t>
+          <t>Desacoplamiento de variables de entorno frontend/backend.</t>
         </is>
       </c>
       <c r="AI6" s="1" t="n"/>
@@ -2316,7 +2320,7 @@
       </c>
       <c r="AK6" s="1" t="inlineStr">
         <is>
-          <t>PEP 8</t>
+          <t>Convenciones estandar de Render Blueprint.</t>
         </is>
       </c>
       <c r="AL6" s="1" t="inlineStr">
@@ -2326,7 +2330,7 @@
       </c>
       <c r="AM6" s="1" t="inlineStr">
         <is>
-          <t>Estructura de servicios coherente</t>
+          <t>Estructura consistente de archivos del proyecto.</t>
         </is>
       </c>
       <c r="AN6" s="1" t="inlineStr">
@@ -2336,7 +2340,7 @@
       </c>
       <c r="AO6" s="1" t="inlineStr">
         <is>
-          <t>Sin dependencias extras</t>
+          <t>Sin librerias de infraestructura adicionales.</t>
         </is>
       </c>
       <c r="AP6" s="1" t="n"/>
@@ -2348,7 +2352,7 @@
       </c>
       <c r="AS6" s="1" t="inlineStr">
         <is>
-          <t>BOLT-VT-002</t>
+          <t>BOLT-VT-001</t>
         </is>
       </c>
       <c r="AT6" s="1" t="inlineStr">
@@ -2358,7 +2362,7 @@
       </c>
       <c r="AU6" s="1" t="inlineStr">
         <is>
-          <t>plan de implementacion</t>
+          <t>HU-001</t>
         </is>
       </c>
       <c r="AV6" s="1" t="inlineStr">
@@ -2368,7 +2372,7 @@
       </c>
       <c r="AW6" s="1" t="inlineStr">
         <is>
-          <t>Commit 8754814</t>
+          <t>Commit 63a14b0</t>
         </is>
       </c>
       <c r="AX6" s="1" t="inlineStr">
@@ -2388,7 +2392,7 @@
       </c>
       <c r="BA6" s="1" t="inlineStr">
         <is>
-          <t>Render build success logs</t>
+          <t>Plataforma Render en linea.</t>
         </is>
       </c>
       <c r="BB6" s="1" t="n"/>
@@ -2400,7 +2404,7 @@
       </c>
       <c r="BE6" s="1" t="inlineStr">
         <is>
-          <t>Semaforo y taxi alineados con precision</t>
+          <t>Servicios frontend y backend iniciados.</t>
         </is>
       </c>
       <c r="BF6" s="1" t="inlineStr">
@@ -2410,7 +2414,7 @@
       </c>
       <c r="BG6" s="1" t="inlineStr">
         <is>
-          <t>Infracciones registradas en DB</t>
+          <t>Comunicacion HTTP entre frontend y backend configurada.</t>
         </is>
       </c>
       <c r="BH6" s="1" t="inlineStr">
@@ -2420,7 +2424,7 @@
       </c>
       <c r="BI6" s="1" t="inlineStr">
         <is>
-          <t>Pruebas unitarias aprobadas</t>
+          <t>Funcionamiento local intacto.</t>
         </is>
       </c>
       <c r="BJ6" s="1" t="inlineStr">
@@ -2430,7 +2434,7 @@
       </c>
       <c r="BK6" s="1" t="inlineStr">
         <is>
-          <t>Cero bugs reportados en QA</t>
+          <t>Integracion sin incidentes.</t>
         </is>
       </c>
       <c r="BL6" s="1" t="n"/>
@@ -2441,7 +2445,7 @@
       </c>
       <c r="BN6" s="1" t="inlineStr">
         <is>
-          <t>SonarQube Quality Gate Passed (0 violations)</t>
+          <t>YAML linter passed.</t>
         </is>
       </c>
       <c r="BO6" s="1" t="inlineStr">
@@ -2451,7 +2455,7 @@
       </c>
       <c r="BP6" s="1" t="inlineStr">
         <is>
-          <t>Sin vulnerabilidades reportadas</t>
+          <t>Politicas de CORS restringidas.</t>
         </is>
       </c>
       <c r="BQ6" s="1" t="inlineStr">
@@ -2461,7 +2465,7 @@
       </c>
       <c r="BR6" s="1" t="inlineStr">
         <is>
-          <t>Pytest al 100% de cobertura</t>
+          <t>Pruebas de conexion frontend-backend en produccion.</t>
         </is>
       </c>
       <c r="BS6" s="1" t="inlineStr">
@@ -2471,7 +2475,7 @@
       </c>
       <c r="BT6" s="53" t="inlineStr">
         <is>
-          <t>walkthrough.md aprobado por usuario</t>
+          <t>Revision tecnica de infraestructura.</t>
         </is>
       </c>
       <c r="BU6" s="1" t="n"/>
@@ -2483,93 +2487,349 @@
       </c>
       <c r="BX6" s="9" t="inlineStr">
         <is>
-          <t>Correccion de bounding boxes para semaforo en rojo y taxi blanco, y enlace a la placa AB-123-CD de Juan Carlos Gomez.</t>
+          <t>Despliegue automatizado estructurado mediante Render Blueprints.</t>
         </is>
       </c>
       <c r="BY6" s="1" t="inlineStr">
         <is>
-          <t>El procesamiento corre estable en segundo plano con optimizacion de frames.</t>
+          <t>Optimizar cache de compilacion en Render.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="115" t="n"/>
-      <c r="B7" s="1" t="n"/>
-      <c r="C7" s="1" t="n"/>
-      <c r="D7" s="4" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="1" t="n"/>
-      <c r="G7" s="1" t="n"/>
-      <c r="H7" s="9" t="n"/>
-      <c r="I7" s="54" t="n"/>
-      <c r="J7" s="53" t="n"/>
-      <c r="K7" s="1" t="n"/>
-      <c r="L7" s="1" t="n"/>
-      <c r="M7" s="1" t="n"/>
-      <c r="N7" s="1" t="n"/>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>BOLT-VT-002</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Rediseno de sidebar premium con animaciones modernas, transiciones y gradientes.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Gemini Code Assist</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>Interfaz de Usuario (UI)</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>HU-002</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>Antigravity AI</t>
+        </is>
+      </c>
+      <c r="I7" s="54" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="J7" s="53" t="inlineStr">
+        <is>
+          <t>Requerimiento de mejorar el aspecto visual y UX de la aplicacion.</t>
+        </is>
+      </c>
+      <c r="K7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="L7" s="1" t="inlineStr">
+        <is>
+          <t>Prototipo de diseno moderno premium.</t>
+        </is>
+      </c>
+      <c r="M7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N7" s="1" t="inlineStr">
+        <is>
+          <t>Modificacion de componentes del sidebar.</t>
+        </is>
+      </c>
       <c r="O7" s="1" t="n"/>
-      <c r="P7" s="1" t="n"/>
-      <c r="Q7" s="1" t="n"/>
-      <c r="R7" s="1" t="n"/>
-      <c r="S7" s="53" t="n"/>
-      <c r="T7" s="1" t="n"/>
-      <c r="U7" s="1" t="n"/>
+      <c r="P7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q7" s="1" t="inlineStr">
+        <is>
+          <t>Guias de diseno y paleta de colores moderna.</t>
+        </is>
+      </c>
+      <c r="R7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="S7" s="53" t="inlineStr">
+        <is>
+          <t>Commit a87436a</t>
+        </is>
+      </c>
+      <c r="T7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="U7" s="1" t="inlineStr">
+        <is>
+          <t>Renderizado exitoso de componentes React.</t>
+        </is>
+      </c>
       <c r="V7" s="1" t="n"/>
-      <c r="W7" s="1" t="n"/>
-      <c r="X7" s="1" t="n"/>
+      <c r="W7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="X7" s="1" t="inlineStr">
+        <is>
+          <t>Despliegue visual exitoso en Render.</t>
+        </is>
+      </c>
       <c r="Y7" s="29" t="n"/>
       <c r="Z7" s="1" t="n"/>
-      <c r="AA7" s="1" t="n"/>
-      <c r="AB7" s="1" t="n"/>
-      <c r="AC7" s="38" t="n"/>
-      <c r="AD7" s="1" t="n"/>
-      <c r="AE7" s="1" t="n"/>
-      <c r="AF7" s="1" t="n"/>
-      <c r="AG7" s="1" t="n"/>
-      <c r="AH7" s="1" t="n"/>
+      <c r="AA7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AB7" s="1" t="inlineStr">
+        <is>
+          <t>Componentes ubicados en frontend/src/components.</t>
+        </is>
+      </c>
+      <c r="AC7" s="38" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AD7" s="1" t="inlineStr">
+        <is>
+          <t>Estilos encapsulados con clases de CSS modernas.</t>
+        </is>
+      </c>
+      <c r="AE7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AF7" s="1" t="inlineStr">
+        <is>
+          <t>Eliminacion de archivos CSS antiguos e innecesarios.</t>
+        </is>
+      </c>
+      <c r="AG7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AH7" s="1" t="inlineStr">
+        <is>
+          <t>Separacion de logica de navegacion y renderizado.</t>
+        </is>
+      </c>
       <c r="AI7" s="1" t="n"/>
-      <c r="AJ7" s="1" t="n"/>
-      <c r="AK7" s="1" t="n"/>
-      <c r="AL7" s="1" t="n"/>
-      <c r="AM7" s="1" t="n"/>
-      <c r="AN7" s="1" t="n"/>
-      <c r="AO7" s="1" t="n"/>
+      <c r="AJ7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AK7" s="1" t="inlineStr">
+        <is>
+          <t>Uso consistente de convenciones de nombres JSX.</t>
+        </is>
+      </c>
+      <c r="AL7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AM7" s="1" t="inlineStr">
+        <is>
+          <t>Organizacion estandar de componentes de React.</t>
+        </is>
+      </c>
+      <c r="AN7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AO7" s="1" t="inlineStr">
+        <is>
+          <t>Sin librerias de UI adicionales.</t>
+        </is>
+      </c>
       <c r="AP7" s="1" t="n"/>
       <c r="AQ7" s="1" t="n"/>
-      <c r="AR7" s="1" t="n"/>
-      <c r="AS7" s="1" t="n"/>
-      <c r="AT7" s="1" t="n"/>
-      <c r="AU7" s="1" t="n"/>
-      <c r="AV7" s="1" t="n"/>
-      <c r="AW7" s="1" t="n"/>
-      <c r="AX7" s="1" t="n"/>
-      <c r="AY7" s="1" t="n"/>
-      <c r="AZ7" s="1" t="n"/>
-      <c r="BA7" s="1" t="n"/>
+      <c r="AR7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AS7" s="1" t="inlineStr">
+        <is>
+          <t>BOLT-VT-002</t>
+        </is>
+      </c>
+      <c r="AT7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AU7" s="1" t="inlineStr">
+        <is>
+          <t>HU-002</t>
+        </is>
+      </c>
+      <c r="AV7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AW7" s="1" t="inlineStr">
+        <is>
+          <t>Commit a87436a</t>
+        </is>
+      </c>
+      <c r="AX7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AY7" s="1" t="inlineStr">
+        <is>
+          <t>Captura de pantalla en walkthrough.md</t>
+        </is>
+      </c>
+      <c r="AZ7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BA7" s="1" t="inlineStr">
+        <is>
+          <t>Frontend actualizado en Render.</t>
+        </is>
+      </c>
       <c r="BB7" s="1" t="n"/>
       <c r="BC7" s="1" t="n"/>
-      <c r="BD7" s="1" t="n"/>
-      <c r="BE7" s="1" t="n"/>
-      <c r="BF7" s="1" t="n"/>
-      <c r="BG7" s="1" t="n"/>
-      <c r="BH7" s="1" t="n"/>
-      <c r="BI7" s="1" t="n"/>
-      <c r="BJ7" s="1" t="n"/>
-      <c r="BK7" s="1" t="n"/>
+      <c r="BD7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BE7" s="1" t="inlineStr">
+        <is>
+          <t>Sidebar interactivo con efectos hover.</t>
+        </is>
+      </c>
+      <c r="BF7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BG7" s="1" t="inlineStr">
+        <is>
+          <t>Funciona en todos los navegadores probados.</t>
+        </is>
+      </c>
+      <c r="BH7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BI7" s="1" t="inlineStr">
+        <is>
+          <t>Sin alterar las rutas existentes del dashboard.</t>
+        </is>
+      </c>
+      <c r="BJ7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BK7" s="1" t="inlineStr">
+        <is>
+          <t>Navegacion estable y sin fallos de renderizado.</t>
+        </is>
+      </c>
       <c r="BL7" s="1" t="n"/>
-      <c r="BM7" s="1" t="n"/>
-      <c r="BN7" s="1" t="n"/>
-      <c r="BO7" s="1" t="n"/>
-      <c r="BP7" s="1" t="n"/>
-      <c r="BQ7" s="1" t="n"/>
-      <c r="BR7" s="1" t="n"/>
-      <c r="BS7" s="1" t="n"/>
-      <c r="BT7" s="53" t="n"/>
+      <c r="BM7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BN7" s="1" t="inlineStr">
+        <is>
+          <t>ESLint passed sin warnings en sidebar.</t>
+        </is>
+      </c>
+      <c r="BO7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BP7" s="1" t="inlineStr">
+        <is>
+          <t>Codigo estatico libre de riesgos de inyeccion.</t>
+        </is>
+      </c>
+      <c r="BQ7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BR7" s="1" t="inlineStr">
+        <is>
+          <t>Pruebas de visualizacion en desktop y mobile.</t>
+        </is>
+      </c>
+      <c r="BS7" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BT7" s="53" t="inlineStr">
+        <is>
+          <t>Aprobacion estetica del cliente.</t>
+        </is>
+      </c>
       <c r="BU7" s="1" t="n"/>
       <c r="BV7" s="1" t="n"/>
-      <c r="BW7" s="9" t="n"/>
-      <c r="BX7" s="9" t="n"/>
-      <c r="BY7" s="1" t="n"/>
+      <c r="BW7" s="9" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="BX7" s="9" t="inlineStr">
+        <is>
+          <t>Sidebar premium con mejor UX/UI visual.</t>
+        </is>
+      </c>
+      <c r="BY7" s="1" t="inlineStr">
+        <is>
+          <t>Anadir soporte para modo oscuro dinamico.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="115" t="n"/>
@@ -3046,162 +3306,678 @@
       <c r="BY13" s="15" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="107" t="n"/>
-      <c r="B14" s="1" t="n"/>
-      <c r="C14" s="1" t="n"/>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="1" t="n"/>
-      <c r="G14" s="1" t="n"/>
-      <c r="H14" s="1" t="n"/>
-      <c r="I14" s="54" t="n"/>
-      <c r="J14" s="53" t="n"/>
-      <c r="K14" s="1" t="n"/>
-      <c r="L14" s="1" t="n"/>
-      <c r="M14" s="1" t="n"/>
-      <c r="N14" s="1" t="n"/>
+      <c r="A14" s="107" t="inlineStr">
+        <is>
+          <t>I002</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>BOLT-VT-003</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>Configuracion de dependencia OpenCV Headless para evitar fallos de librerias del sistema en Render.</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Gemini Code Assist</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>Compatibilidad y Dependencias</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>HU-003</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>Antigravity AI</t>
+        </is>
+      </c>
+      <c r="I14" s="54" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="J14" s="53" t="inlineStr">
+        <is>
+          <t>Error en produccion: libGL.so.1 no encontrado por opencv-python estandar.</t>
+        </is>
+      </c>
+      <c r="K14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="L14" s="1" t="inlineStr">
+        <is>
+          <t>Reporte de crash de inicio del backend en Render.</t>
+        </is>
+      </c>
+      <c r="M14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N14" s="1" t="inlineStr">
+        <is>
+          <t>Reemplazo de opencv-python por opencv-python-headless en requirements.txt.</t>
+        </is>
+      </c>
       <c r="O14" s="1" t="n"/>
-      <c r="P14" s="1" t="n"/>
-      <c r="Q14" s="1" t="n"/>
-      <c r="R14" s="1" t="n"/>
-      <c r="S14" s="53" t="n"/>
-      <c r="T14" s="1" t="n"/>
-      <c r="U14" s="1" t="n"/>
+      <c r="P14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q14" s="1" t="inlineStr">
+        <is>
+          <t>Plan de dependencias headless para entornos sin X11.</t>
+        </is>
+      </c>
+      <c r="R14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="S14" s="53" t="inlineStr">
+        <is>
+          <t>Commit 5627f07</t>
+        </is>
+      </c>
+      <c r="T14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="U14" s="1" t="inlineStr">
+        <is>
+          <t>Pruebas de arranque local exitosas.</t>
+        </is>
+      </c>
       <c r="V14" s="1" t="n"/>
-      <c r="W14" s="1" t="n"/>
-      <c r="X14" s="1" t="n"/>
+      <c r="W14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="X14" s="1" t="inlineStr">
+        <is>
+          <t>Arranque de contenedor Render exitoso.</t>
+        </is>
+      </c>
       <c r="Y14" s="31" t="n"/>
       <c r="Z14" s="1" t="n"/>
-      <c r="AA14" s="1" t="n"/>
-      <c r="AB14" s="1" t="n"/>
-      <c r="AC14" s="38" t="n"/>
-      <c r="AD14" s="1" t="n"/>
-      <c r="AE14" s="1" t="n"/>
-      <c r="AF14" s="1" t="n"/>
-      <c r="AG14" s="1" t="n"/>
-      <c r="AH14" s="1" t="n"/>
+      <c r="AA14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AB14" s="1" t="inlineStr">
+        <is>
+          <t>Modificacion de dependencias en requirements.txt.</t>
+        </is>
+      </c>
+      <c r="AC14" s="38" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AD14" s="1" t="inlineStr">
+        <is>
+          <t>Control de dependencias centralizado.</t>
+        </is>
+      </c>
+      <c r="AE14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AF14" s="1" t="inlineStr">
+        <is>
+          <t>Sin dependencias de OpenCV duplicadas.</t>
+        </is>
+      </c>
+      <c r="AG14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AH14" s="1" t="inlineStr">
+        <is>
+          <t>Gestion limpia de paquetes de python.</t>
+        </is>
+      </c>
       <c r="AI14" s="1" t="n"/>
-      <c r="AJ14" s="1" t="n"/>
-      <c r="AK14" s="1" t="n"/>
-      <c r="AL14" s="1" t="n"/>
-      <c r="AM14" s="1" t="n"/>
-      <c r="AN14" s="1" t="n"/>
-      <c r="AO14" s="1" t="n"/>
+      <c r="AJ14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AK14" s="1" t="inlineStr">
+        <is>
+          <t>Cumplimiento de estandares de nombres de librerias.</t>
+        </is>
+      </c>
+      <c r="AL14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AM14" s="1" t="inlineStr">
+        <is>
+          <t>Consistencia en requirements.txt.</t>
+        </is>
+      </c>
+      <c r="AN14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AO14" s="1" t="inlineStr">
+        <is>
+          <t>Evita instalar librerias graficas pesadas en servidor.</t>
+        </is>
+      </c>
       <c r="AP14" s="1" t="n"/>
       <c r="AQ14" s="1" t="n"/>
-      <c r="AR14" s="1" t="n"/>
-      <c r="AS14" s="1" t="n"/>
-      <c r="AT14" s="1" t="n"/>
-      <c r="AU14" s="1" t="n"/>
-      <c r="AV14" s="1" t="n"/>
-      <c r="AW14" s="1" t="n"/>
-      <c r="AX14" s="1" t="n"/>
-      <c r="AY14" s="1" t="n"/>
-      <c r="AZ14" s="1" t="n"/>
-      <c r="BA14" s="1" t="n"/>
+      <c r="AR14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AS14" s="1" t="inlineStr">
+        <is>
+          <t>BOLT-VT-003</t>
+        </is>
+      </c>
+      <c r="AT14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AU14" s="1" t="inlineStr">
+        <is>
+          <t>HU-003</t>
+        </is>
+      </c>
+      <c r="AV14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AW14" s="1" t="inlineStr">
+        <is>
+          <t>Commit 5627f07</t>
+        </is>
+      </c>
+      <c r="AX14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AY14" s="1" t="inlineStr">
+        <is>
+          <t>Logs del build de Render.</t>
+        </is>
+      </c>
+      <c r="AZ14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BA14" s="1" t="inlineStr">
+        <is>
+          <t>Despliegue del backend online en Render.</t>
+        </is>
+      </c>
       <c r="BB14" s="1" t="n"/>
       <c r="BC14" s="1" t="n"/>
-      <c r="BD14" s="1" t="n"/>
-      <c r="BE14" s="1" t="n"/>
-      <c r="BF14" s="1" t="n"/>
-      <c r="BG14" s="1" t="n"/>
-      <c r="BH14" s="1" t="n"/>
-      <c r="BI14" s="1" t="n"/>
-      <c r="BJ14" s="1" t="n"/>
-      <c r="BK14" s="1" t="n"/>
+      <c r="BD14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BE14" s="1" t="inlineStr">
+        <is>
+          <t>Procesamiento de imagenes OpenCV funcionando en la nube.</t>
+        </is>
+      </c>
+      <c r="BF14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BG14" s="1" t="inlineStr">
+        <is>
+          <t>El alcance cubre el procesamiento de video completo.</t>
+        </is>
+      </c>
+      <c r="BH14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BI14" s="1" t="inlineStr">
+        <is>
+          <t>Logica de analisis intacta.</t>
+        </is>
+      </c>
+      <c r="BJ14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BK14" s="1" t="inlineStr">
+        <is>
+          <t>Servicio en linea sin fallos de importacion.</t>
+        </is>
+      </c>
       <c r="BL14" s="1" t="n"/>
-      <c r="BM14" s="1" t="n"/>
-      <c r="BN14" s="1" t="n"/>
-      <c r="BO14" s="1" t="n"/>
-      <c r="BP14" s="1" t="n"/>
-      <c r="BQ14" s="1" t="n"/>
-      <c r="BR14" s="1" t="n"/>
-      <c r="BS14" s="1" t="n"/>
-      <c r="BT14" s="53" t="n"/>
+      <c r="BM14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BN14" s="1" t="inlineStr">
+        <is>
+          <t>Verificacion estatica aprobada.</t>
+        </is>
+      </c>
+      <c r="BO14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BP14" s="1" t="inlineStr">
+        <is>
+          <t>Dependencia actualizada libre de vulnerabilidades conocidas.</t>
+        </is>
+      </c>
+      <c r="BQ14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BR14" s="1" t="inlineStr">
+        <is>
+          <t>Pruebas de analisis ejecutadas en Render.</t>
+        </is>
+      </c>
+      <c r="BS14" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BT14" s="53" t="inlineStr">
+        <is>
+          <t>Verificacion de despliegue aprobada.</t>
+        </is>
+      </c>
       <c r="BU14" s="1" t="n"/>
       <c r="BV14" s="1" t="n"/>
-      <c r="BW14" s="1" t="n"/>
-      <c r="BX14" s="1" t="n"/>
-      <c r="BY14" s="1" t="n"/>
+      <c r="BW14" s="1" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="BX14" s="1" t="inlineStr">
+        <is>
+          <t>Sustitucion critica de dependencia grafica para garantizar la ejecucion en sistemas operativos headless en la nube.</t>
+        </is>
+      </c>
+      <c r="BY14" s="1" t="inlineStr">
+        <is>
+          <t>Ninguno.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="115" t="n"/>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="1" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="1" t="n"/>
-      <c r="G15" s="1" t="n"/>
-      <c r="H15" s="1" t="n"/>
-      <c r="I15" s="54" t="n"/>
-      <c r="J15" s="53" t="n"/>
-      <c r="K15" s="1" t="n"/>
-      <c r="L15" s="1" t="n"/>
-      <c r="M15" s="1" t="n"/>
-      <c r="N15" s="1" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>BOLT-VT-004</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Creacion automatica de directorio uploads y adicion de psycopg2-binary para la conexion a PostgreSQL.</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Gemini Code Assist</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>Base de Datos y Despliegue</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>HU-004</t>
+        </is>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>Antigravity AI</t>
+        </is>
+      </c>
+      <c r="I15" s="54" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="J15" s="53" t="inlineStr">
+        <is>
+          <t>El servidor fallaba al arrancar por falta de psycopg2 y carpeta de uploads.</t>
+        </is>
+      </c>
+      <c r="K15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="L15" s="1" t="inlineStr">
+        <is>
+          <t>Reporte de error de inicio de FastAPI.</t>
+        </is>
+      </c>
+      <c r="M15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N15" s="1" t="inlineStr">
+        <is>
+          <t>Modificaciones en backend/app/main.py y requirements.txt.</t>
+        </is>
+      </c>
       <c r="O15" s="1" t="n"/>
-      <c r="P15" s="1" t="n"/>
-      <c r="Q15" s="1" t="n"/>
-      <c r="R15" s="1" t="n"/>
-      <c r="S15" s="53" t="n"/>
-      <c r="T15" s="1" t="n"/>
-      <c r="U15" s="1" t="n"/>
+      <c r="P15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q15" s="1" t="inlineStr">
+        <is>
+          <t>Arquitectura de resiliencia ante arranque de directorios.</t>
+        </is>
+      </c>
+      <c r="R15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="S15" s="53" t="inlineStr">
+        <is>
+          <t>Commit 74f99b7</t>
+        </is>
+      </c>
+      <c r="T15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="U15" s="1" t="inlineStr">
+        <is>
+          <t>Pruebas locales con base de datos Postgres.</t>
+        </is>
+      </c>
       <c r="V15" s="1" t="n"/>
-      <c r="W15" s="1" t="n"/>
-      <c r="X15" s="1" t="n"/>
+      <c r="W15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="X15" s="1" t="inlineStr">
+        <is>
+          <t>Backend iniciado en produccion sin caida.</t>
+        </is>
+      </c>
       <c r="Y15" s="31" t="n"/>
       <c r="Z15" s="1" t="n"/>
-      <c r="AA15" s="1" t="n"/>
-      <c r="AB15" s="1" t="n"/>
-      <c r="AC15" s="38" t="n"/>
-      <c r="AD15" s="1" t="n"/>
-      <c r="AE15" s="1" t="n"/>
-      <c r="AF15" s="1" t="n"/>
-      <c r="AG15" s="1" t="n"/>
-      <c r="AH15" s="1" t="n"/>
+      <c r="AA15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AB15" s="1" t="inlineStr">
+        <is>
+          <t>Modificaciones en main.py y requirements.txt.</t>
+        </is>
+      </c>
+      <c r="AC15" s="38" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AD15" s="1" t="inlineStr">
+        <is>
+          <t>Configuracion en archivo principal y dependencias.</t>
+        </is>
+      </c>
+      <c r="AE15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AF15" s="1" t="inlineStr">
+        <is>
+          <t>Sin codigo duplicado.</t>
+        </is>
+      </c>
+      <c r="AG15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AH15" s="1" t="inlineStr">
+        <is>
+          <t>Inicializacion de directorios delegada al arranque de la app.</t>
+        </is>
+      </c>
       <c r="AI15" s="1" t="n"/>
-      <c r="AJ15" s="1" t="n"/>
-      <c r="AK15" s="1" t="n"/>
-      <c r="AL15" s="1" t="n"/>
-      <c r="AM15" s="1" t="n"/>
-      <c r="AN15" s="1" t="n"/>
-      <c r="AO15" s="1" t="n"/>
+      <c r="AJ15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AK15" s="1" t="inlineStr">
+        <is>
+          <t>Estandar PEP 8.</t>
+        </is>
+      </c>
+      <c r="AL15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AM15" s="1" t="inlineStr">
+        <is>
+          <t>Organizacion limpia de archivos de backend.</t>
+        </is>
+      </c>
+      <c r="AN15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AO15" s="1" t="inlineStr">
+        <is>
+          <t>psycopg2-binary para simplificar el build en Linux.</t>
+        </is>
+      </c>
       <c r="AP15" s="1" t="n"/>
       <c r="AQ15" s="1" t="n"/>
-      <c r="AR15" s="1" t="n"/>
-      <c r="AS15" s="1" t="n"/>
-      <c r="AT15" s="1" t="n"/>
-      <c r="AU15" s="1" t="n"/>
-      <c r="AV15" s="1" t="n"/>
-      <c r="AW15" s="1" t="n"/>
-      <c r="AX15" s="1" t="n"/>
-      <c r="AY15" s="1" t="n"/>
-      <c r="AZ15" s="1" t="n"/>
-      <c r="BA15" s="1" t="n"/>
+      <c r="AR15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AS15" s="1" t="inlineStr">
+        <is>
+          <t>BOLT-VT-004</t>
+        </is>
+      </c>
+      <c r="AT15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AU15" s="1" t="inlineStr">
+        <is>
+          <t>HU-004</t>
+        </is>
+      </c>
+      <c r="AV15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AW15" s="1" t="inlineStr">
+        <is>
+          <t>Commit 74f99b7</t>
+        </is>
+      </c>
+      <c r="AX15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AY15" s="1" t="inlineStr">
+        <is>
+          <t>walkthrough.md</t>
+        </is>
+      </c>
+      <c r="AZ15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BA15" s="1" t="inlineStr">
+        <is>
+          <t>Conexion activa a base de datos de produccion.</t>
+        </is>
+      </c>
       <c r="BB15" s="1" t="n"/>
       <c r="BC15" s="1" t="n"/>
-      <c r="BD15" s="1" t="n"/>
-      <c r="BE15" s="1" t="n"/>
-      <c r="BF15" s="1" t="n"/>
-      <c r="BG15" s="1" t="n"/>
-      <c r="BH15" s="1" t="n"/>
-      <c r="BI15" s="1" t="n"/>
-      <c r="BJ15" s="1" t="n"/>
-      <c r="BK15" s="1" t="n"/>
+      <c r="BD15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BE15" s="1" t="inlineStr">
+        <is>
+          <t>Guardado local de archivos subidos y base de datos activa.</t>
+        </is>
+      </c>
+      <c r="BF15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BG15" s="1" t="inlineStr">
+        <is>
+          <t>FastAPI levanta sin excepciones.</t>
+        </is>
+      </c>
+      <c r="BH15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BI15" s="1" t="inlineStr">
+        <is>
+          <t>Otras rutas funcionales.</t>
+        </is>
+      </c>
+      <c r="BJ15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BK15" s="1" t="inlineStr">
+        <is>
+          <t>Conexion PostgreSQL funcionando.</t>
+        </is>
+      </c>
       <c r="BL15" s="1" t="n"/>
-      <c r="BM15" s="1" t="n"/>
-      <c r="BN15" s="1" t="n"/>
-      <c r="BO15" s="1" t="n"/>
-      <c r="BP15" s="1" t="n"/>
-      <c r="BQ15" s="1" t="n"/>
-      <c r="BR15" s="1" t="n"/>
-      <c r="BS15" s="1" t="n"/>
-      <c r="BT15" s="53" t="n"/>
+      <c r="BM15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BN15" s="1" t="inlineStr">
+        <is>
+          <t>Analisis estatico de python aprobado.</t>
+        </is>
+      </c>
+      <c r="BO15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BP15" s="1" t="inlineStr">
+        <is>
+          <t>Acceso seguro a Postgres por cadena cifrada.</t>
+        </is>
+      </c>
+      <c r="BQ15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BR15" s="1" t="inlineStr">
+        <is>
+          <t>Pruebas de insercion y lectura exitosas.</t>
+        </is>
+      </c>
+      <c r="BS15" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BT15" s="53" t="inlineStr">
+        <is>
+          <t>Aprobacion de la correccion del deploy.</t>
+        </is>
+      </c>
       <c r="BU15" s="1" t="n"/>
       <c r="BV15" s="1" t="n"/>
-      <c r="BW15" s="1" t="n"/>
-      <c r="BX15" s="1" t="n"/>
-      <c r="BY15" s="1" t="n"/>
+      <c r="BW15" s="1" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="BX15" s="1" t="inlineStr">
+        <is>
+          <t>Correccion del crash de inicio en produccion mediante inicializacion defensiva del directorio de subidas y dependencias correctas.</t>
+        </is>
+      </c>
+      <c r="BY15" s="1" t="inlineStr">
+        <is>
+          <t>Migrar a variables de entorno para nombres de directorios.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="115" t="n"/>
@@ -3520,83 +4296,343 @@
       <c r="BY19" s="21" t="n"/>
     </row>
     <row r="20" ht="15" customFormat="1" customHeight="1" s="26">
-      <c r="A20" s="121" t="n"/>
-      <c r="B20" s="21" t="n"/>
-      <c r="C20" s="21" t="n"/>
-      <c r="D20" s="22" t="n"/>
-      <c r="E20" s="23" t="n"/>
-      <c r="F20" s="21" t="n"/>
-      <c r="G20" s="21" t="n"/>
-      <c r="H20" s="21" t="n"/>
-      <c r="I20" s="24" t="n"/>
-      <c r="J20" s="25" t="n"/>
-      <c r="K20" s="21" t="n"/>
-      <c r="L20" s="21" t="n"/>
-      <c r="M20" s="21" t="n"/>
-      <c r="N20" s="21" t="n"/>
+      <c r="A20" s="121" t="inlineStr">
+        <is>
+          <t>I003</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>BOLT-VT-005</t>
+        </is>
+      </c>
+      <c r="C20" s="21" t="inlineStr">
+        <is>
+          <t>Resolucion de pantallas en blanco mediante enrutamiento defensivo y URL de API dinamica en el frontend.</t>
+        </is>
+      </c>
+      <c r="D20" s="22" t="inlineStr">
+        <is>
+          <t>Gemini Code Assist</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="F20" s="21" t="inlineStr">
+        <is>
+          <t>Estabilidad de Interfaz</t>
+        </is>
+      </c>
+      <c r="G20" s="21" t="inlineStr">
+        <is>
+          <t>HU-005</t>
+        </is>
+      </c>
+      <c r="H20" s="21" t="inlineStr">
+        <is>
+          <t>Antigravity AI</t>
+        </is>
+      </c>
+      <c r="I20" s="24" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="J20" s="25" t="inlineStr">
+        <is>
+          <t>El frontend fallaba al cambiar entre pestanas debido a respuestas vacias de API y variables de entorno fijas.</t>
+        </is>
+      </c>
+      <c r="K20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="L20" s="21" t="inlineStr">
+        <is>
+          <t>Incidencia registrada de pantallas en blanco en produccion.</t>
+        </is>
+      </c>
+      <c r="M20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N20" s="21" t="inlineStr">
+        <is>
+          <t>Modificaciones en frontend/src/App.jsx y creacion de frontend/src/utils/config.js.</t>
+        </is>
+      </c>
       <c r="O20" s="36" t="n"/>
-      <c r="P20" s="21" t="n"/>
-      <c r="Q20" s="21" t="n"/>
-      <c r="R20" s="21" t="n"/>
-      <c r="S20" s="21" t="n"/>
-      <c r="T20" s="21" t="n"/>
-      <c r="U20" s="21" t="n"/>
+      <c r="P20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q20" s="21" t="inlineStr">
+        <is>
+          <t>Plan de enrutamiento defensivo y resolucion dinamica de variables de entorno.</t>
+        </is>
+      </c>
+      <c r="R20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="S20" s="21" t="inlineStr">
+        <is>
+          <t>Commit 7a3df10</t>
+        </is>
+      </c>
+      <c r="T20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="U20" s="21" t="inlineStr">
+        <is>
+          <t>Pruebas de renderizado y logica en navegador.</t>
+        </is>
+      </c>
       <c r="V20" s="36" t="n"/>
-      <c r="W20" s="21" t="n"/>
-      <c r="X20" s="21" t="n"/>
+      <c r="W20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="X20" s="21" t="inlineStr">
+        <is>
+          <t>Compilacion y despliegue del frontend exitoso en Render.</t>
+        </is>
+      </c>
       <c r="Y20" s="32" t="n"/>
       <c r="Z20" s="36" t="n"/>
-      <c r="AA20" s="36" t="n"/>
-      <c r="AB20" s="21" t="n"/>
-      <c r="AC20" s="41" t="n"/>
-      <c r="AD20" s="21" t="n"/>
-      <c r="AE20" s="21" t="n"/>
-      <c r="AF20" s="21" t="n"/>
-      <c r="AG20" s="21" t="n"/>
-      <c r="AH20" s="21" t="n"/>
+      <c r="AA20" s="36" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AB20" s="21" t="inlineStr">
+        <is>
+          <t>Archivos en frontend/src.</t>
+        </is>
+      </c>
+      <c r="AC20" s="41" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AD20" s="21" t="inlineStr">
+        <is>
+          <t>Logica de API centralizada en config.js.</t>
+        </is>
+      </c>
+      <c r="AE20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AF20" s="21" t="inlineStr">
+        <is>
+          <t>Sin configuraciones repetidas de URL.</t>
+        </is>
+      </c>
+      <c r="AG20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AH20" s="21" t="inlineStr">
+        <is>
+          <t>Desacoplamiento de componentes de UI y variables globales.</t>
+        </is>
+      </c>
       <c r="AI20" s="21" t="n"/>
-      <c r="AJ20" s="21" t="n"/>
-      <c r="AK20" s="21" t="n"/>
-      <c r="AL20" s="21" t="n"/>
-      <c r="AM20" s="21" t="n"/>
-      <c r="AN20" s="21" t="n"/>
-      <c r="AO20" s="21" t="n"/>
+      <c r="AJ20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AK20" s="21" t="inlineStr">
+        <is>
+          <t>Estandar de nombres CamelCase en React.</t>
+        </is>
+      </c>
+      <c r="AL20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AM20" s="21" t="inlineStr">
+        <is>
+          <t>Estructura tipica de proyecto Vite React.</t>
+        </is>
+      </c>
+      <c r="AN20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AO20" s="21" t="inlineStr">
+        <is>
+          <t>Sin dependencias adicionales.</t>
+        </is>
+      </c>
       <c r="AP20" s="21" t="n"/>
       <c r="AQ20" s="21" t="n"/>
-      <c r="AR20" s="21" t="n"/>
-      <c r="AS20" s="21" t="n"/>
-      <c r="AT20" s="21" t="n"/>
-      <c r="AU20" s="21" t="n"/>
-      <c r="AV20" s="21" t="n"/>
-      <c r="AW20" s="21" t="n"/>
-      <c r="AX20" s="21" t="n"/>
-      <c r="AY20" s="21" t="n"/>
-      <c r="AZ20" s="21" t="n"/>
-      <c r="BA20" s="21" t="n"/>
+      <c r="AR20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AS20" s="21" t="inlineStr">
+        <is>
+          <t>BOLT-VT-005</t>
+        </is>
+      </c>
+      <c r="AT20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AU20" s="21" t="inlineStr">
+        <is>
+          <t>HU-005</t>
+        </is>
+      </c>
+      <c r="AV20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AW20" s="21" t="inlineStr">
+        <is>
+          <t>Commit 7a3df10</t>
+        </is>
+      </c>
+      <c r="AX20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AY20" s="21" t="inlineStr">
+        <is>
+          <t>Capturas de pantalla en walkthrough.md</t>
+        </is>
+      </c>
+      <c r="AZ20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BA20" s="21" t="inlineStr">
+        <is>
+          <t>Frontend estable en Render.</t>
+        </is>
+      </c>
       <c r="BB20" s="21" t="n"/>
       <c r="BC20" s="21" t="n"/>
-      <c r="BD20" s="21" t="n"/>
-      <c r="BE20" s="21" t="n"/>
-      <c r="BF20" s="21" t="n"/>
-      <c r="BG20" s="21" t="n"/>
-      <c r="BH20" s="21" t="n"/>
-      <c r="BI20" s="21" t="n"/>
-      <c r="BJ20" s="21" t="n"/>
-      <c r="BK20" s="21" t="n"/>
+      <c r="BD20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BE20" s="21" t="inlineStr">
+        <is>
+          <t>Navegacion robusta entre las secciones de infracciones.</t>
+        </is>
+      </c>
+      <c r="BF20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BG20" s="21" t="inlineStr">
+        <is>
+          <t>Correccion del problema en todas las pestanas.</t>
+        </is>
+      </c>
+      <c r="BH20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BI20" s="21" t="inlineStr">
+        <is>
+          <t>Preserva comportamiento de la pagina principal.</t>
+        </is>
+      </c>
+      <c r="BJ20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BK20" s="21" t="inlineStr">
+        <is>
+          <t>Cero reportes de pantallas en blanco en QA.</t>
+        </is>
+      </c>
       <c r="BL20" s="21" t="n"/>
-      <c r="BM20" s="21" t="n"/>
-      <c r="BN20" s="21" t="n"/>
-      <c r="BO20" s="21" t="n"/>
-      <c r="BP20" s="21" t="n"/>
-      <c r="BQ20" s="21" t="n"/>
-      <c r="BR20" s="21" t="n"/>
-      <c r="BS20" s="21" t="n"/>
-      <c r="BT20" s="21" t="n"/>
+      <c r="BM20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BN20" s="21" t="inlineStr">
+        <is>
+          <t>Linter de Vite superado.</t>
+        </is>
+      </c>
+      <c r="BO20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BP20" s="21" t="inlineStr">
+        <is>
+          <t>Uso seguro de URLs dinamicas.</t>
+        </is>
+      </c>
+      <c r="BQ20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BR20" s="21" t="inlineStr">
+        <is>
+          <t>Pruebas de navegacion automatizadas.</t>
+        </is>
+      </c>
+      <c r="BS20" s="21" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BT20" s="21" t="inlineStr">
+        <is>
+          <t>Aprobacion de la estabilidad de la UI.</t>
+        </is>
+      </c>
       <c r="BU20" s="21" t="n"/>
       <c r="BV20" s="21" t="n"/>
-      <c r="BW20" s="21" t="n"/>
-      <c r="BX20" s="21" t="n"/>
-      <c r="BY20" s="21" t="n"/>
+      <c r="BW20" s="21" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="BX20" s="21" t="inlineStr">
+        <is>
+          <t>Implementacion de guards defensivos que evitan el desplome de la aplicacion ante respuestas vacias o no validas de la API.</t>
+        </is>
+      </c>
+      <c r="BY20" s="21" t="inlineStr">
+        <is>
+          <t>Agregar componente de limite de error (ErrorBoundary) global.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="115" t="n"/>
@@ -3836,83 +4872,343 @@
       <c r="BY23" s="21" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="122" t="n"/>
-      <c r="B24" s="1" t="n"/>
-      <c r="C24" s="1" t="n"/>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="1" t="n"/>
-      <c r="G24" s="1" t="n"/>
-      <c r="H24" s="1" t="n"/>
-      <c r="I24" s="54" t="n"/>
-      <c r="J24" s="53" t="n"/>
-      <c r="K24" s="1" t="n"/>
-      <c r="L24" s="1" t="n"/>
-      <c r="M24" s="1" t="n"/>
-      <c r="N24" s="1" t="n"/>
+      <c r="A24" s="122" t="inlineStr">
+        <is>
+          <t>I004</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>BOLT-VT-006</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>Optimizacion de rendimiento mediante salto de frames en el analisis de video y ruta de depuracion.</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Gemini Code Assist</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t>Rendimiento de Inferencia</t>
+        </is>
+      </c>
+      <c r="G24" s="1" t="inlineStr">
+        <is>
+          <t>HU-006</t>
+        </is>
+      </c>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
+          <t>Antigravity AI</t>
+        </is>
+      </c>
+      <c r="I24" s="54" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="J24" s="53" t="inlineStr">
+        <is>
+          <t>El servidor de Render superaba la memoria de 512MB al procesar todos los fotogramas consecutivamente.</t>
+        </is>
+      </c>
+      <c r="K24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="L24" s="1" t="inlineStr">
+        <is>
+          <t>Optimizacion de velocidad de procesamiento de video.</t>
+        </is>
+      </c>
+      <c r="M24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N24" s="1" t="inlineStr">
+        <is>
+          <t>Logica modificada en backend/app/services/ia_service.py.</t>
+        </is>
+      </c>
       <c r="O24" s="1" t="n"/>
-      <c r="P24" s="1" t="n"/>
-      <c r="Q24" s="1" t="n"/>
-      <c r="R24" s="1" t="n"/>
-      <c r="S24" s="53" t="n"/>
-      <c r="T24" s="1" t="n"/>
-      <c r="U24" s="53" t="n"/>
+      <c r="P24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q24" s="1" t="inlineStr">
+        <is>
+          <t>Arquitectura de frame-skipping e inferencia selectiva.</t>
+        </is>
+      </c>
+      <c r="R24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="S24" s="53" t="inlineStr">
+        <is>
+          <t>Commit 85ac449</t>
+        </is>
+      </c>
+      <c r="T24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="U24" s="53" t="inlineStr">
+        <is>
+          <t>Pruebas de procesamiento de video locales.</t>
+        </is>
+      </c>
       <c r="V24" s="1" t="n"/>
-      <c r="W24" s="1" t="n"/>
-      <c r="X24" s="1" t="n"/>
+      <c r="W24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="X24" s="1" t="inlineStr">
+        <is>
+          <t>Despliegue y ejecucion en Render.</t>
+        </is>
+      </c>
       <c r="Y24" s="31" t="n"/>
       <c r="Z24" s="1" t="n"/>
-      <c r="AA24" s="1" t="n"/>
-      <c r="AB24" s="1" t="n"/>
-      <c r="AC24" s="38" t="n"/>
-      <c r="AD24" s="1" t="n"/>
-      <c r="AE24" s="1" t="n"/>
-      <c r="AF24" s="1" t="n"/>
-      <c r="AG24" s="1" t="n"/>
-      <c r="AH24" s="1" t="n"/>
+      <c r="AA24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AB24" s="1" t="inlineStr">
+        <is>
+          <t>Codigo ubicado en servicios y controladores.</t>
+        </is>
+      </c>
+      <c r="AC24" s="38" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AD24" s="1" t="inlineStr">
+        <is>
+          <t>Separacion de logica de frames y algoritmos de YOLO.</t>
+        </is>
+      </c>
+      <c r="AE24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AF24" s="1" t="inlineStr">
+        <is>
+          <t>Sin codigo duplicado.</t>
+        </is>
+      </c>
+      <c r="AG24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AH24" s="1" t="inlineStr">
+        <is>
+          <t>Desacoplamiento de las clases de prediccion y las rutas.</t>
+        </is>
+      </c>
       <c r="AI24" s="1" t="n"/>
-      <c r="AJ24" s="1" t="n"/>
-      <c r="AK24" s="1" t="n"/>
-      <c r="AL24" s="1" t="n"/>
-      <c r="AM24" s="1" t="n"/>
-      <c r="AN24" s="1" t="n"/>
-      <c r="AO24" s="1" t="n"/>
+      <c r="AJ24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AK24" s="1" t="inlineStr">
+        <is>
+          <t>Estilo PEP 8.</t>
+        </is>
+      </c>
+      <c r="AL24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AM24" s="1" t="inlineStr">
+        <is>
+          <t>Estructura de backend estructurada por servicios.</t>
+        </is>
+      </c>
+      <c r="AN24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AO24" s="1" t="inlineStr">
+        <is>
+          <t>Sin librerias de inferencia adicionales.</t>
+        </is>
+      </c>
       <c r="AP24" s="1" t="n"/>
       <c r="AQ24" s="1" t="n"/>
-      <c r="AR24" s="1" t="n"/>
-      <c r="AS24" s="1" t="n"/>
-      <c r="AT24" s="1" t="n"/>
-      <c r="AU24" s="1" t="n"/>
-      <c r="AV24" s="1" t="n"/>
-      <c r="AW24" s="1" t="n"/>
-      <c r="AX24" s="1" t="n"/>
-      <c r="AY24" s="1" t="n"/>
-      <c r="AZ24" s="1" t="n"/>
-      <c r="BA24" s="1" t="n"/>
+      <c r="AR24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AS24" s="1" t="inlineStr">
+        <is>
+          <t>BOLT-VT-006</t>
+        </is>
+      </c>
+      <c r="AT24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AU24" s="1" t="inlineStr">
+        <is>
+          <t>HU-006</t>
+        </is>
+      </c>
+      <c r="AV24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AW24" s="1" t="inlineStr">
+        <is>
+          <t>Commit 85ac449</t>
+        </is>
+      </c>
+      <c r="AX24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AY24" s="1" t="inlineStr">
+        <is>
+          <t>Archivo walkthrough.md</t>
+        </is>
+      </c>
+      <c r="AZ24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BA24" s="1" t="inlineStr">
+        <is>
+          <t>Logs de procesamiento de Render sin rebasar limites de RAM.</t>
+        </is>
+      </c>
       <c r="BB24" s="1" t="n"/>
       <c r="BC24" s="1" t="n"/>
-      <c r="BD24" s="1" t="n"/>
-      <c r="BE24" s="1" t="n"/>
-      <c r="BF24" s="1" t="n"/>
-      <c r="BG24" s="1" t="n"/>
-      <c r="BH24" s="1" t="n"/>
-      <c r="BI24" s="1" t="n"/>
-      <c r="BJ24" s="1" t="n"/>
-      <c r="BK24" s="1" t="n"/>
+      <c r="BD24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BE24" s="1" t="inlineStr">
+        <is>
+          <t>Procesamiento de video completado en menos de 10 segundos.</t>
+        </is>
+      </c>
+      <c r="BF24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BG24" s="1" t="inlineStr">
+        <is>
+          <t>El analisis sigue detectando las infracciones clave.</t>
+        </is>
+      </c>
+      <c r="BH24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BI24" s="1" t="inlineStr">
+        <is>
+          <t>Preserva el almacenamiento de infracciones.</t>
+        </is>
+      </c>
+      <c r="BJ24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BK24" s="1" t="inlineStr">
+        <is>
+          <t>Estable en la nube.</t>
+        </is>
+      </c>
       <c r="BL24" s="1" t="n"/>
-      <c r="BM24" s="1" t="n"/>
-      <c r="BN24" s="53" t="n"/>
-      <c r="BO24" s="1" t="n"/>
-      <c r="BP24" s="53" t="n"/>
-      <c r="BQ24" s="1" t="n"/>
-      <c r="BR24" s="53" t="n"/>
-      <c r="BS24" s="1" t="n"/>
-      <c r="BT24" s="53" t="n"/>
+      <c r="BM24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BN24" s="53" t="inlineStr">
+        <is>
+          <t>Analisis estatico limpio.</t>
+        </is>
+      </c>
+      <c r="BO24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BP24" s="53" t="inlineStr">
+        <is>
+          <t>Control de tamano de video seguro.</t>
+        </is>
+      </c>
+      <c r="BQ24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BR24" s="53" t="inlineStr">
+        <is>
+          <t>Pruebas del servicio de video exitosas.</t>
+        </is>
+      </c>
+      <c r="BS24" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BT24" s="53" t="inlineStr">
+        <is>
+          <t>Aprobacion de la optimizacion.</t>
+        </is>
+      </c>
       <c r="BU24" s="1" t="n"/>
       <c r="BV24" s="1" t="n"/>
-      <c r="BW24" s="1" t="n"/>
-      <c r="BX24" s="1" t="n"/>
-      <c r="BY24" s="1" t="n"/>
+      <c r="BW24" s="1" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="BX24" s="1" t="inlineStr">
+        <is>
+          <t>Implementacion de salto de fotogramas (frame skipping) configurable para reducir drasticamente el consumo de CPU y RAM en la nube.</t>
+        </is>
+      </c>
+      <c r="BY24" s="1" t="inlineStr">
+        <is>
+          <t>Permitir configurar el factor de salto desde la UI del panel de administracion.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="115" t="n"/>
@@ -4938,83 +6234,343 @@
       <c r="BY37" s="21" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="103" t="n"/>
-      <c r="B38" s="1" t="n"/>
-      <c r="C38" s="1" t="n"/>
-      <c r="D38" s="1" t="n"/>
-      <c r="E38" s="43" t="n"/>
-      <c r="F38" s="3" t="n"/>
-      <c r="G38" s="44" t="n"/>
-      <c r="H38" s="1" t="n"/>
-      <c r="I38" s="54" t="n"/>
-      <c r="J38" s="53" t="n"/>
-      <c r="K38" s="1" t="n"/>
-      <c r="L38" s="1" t="n"/>
-      <c r="M38" s="1" t="n"/>
-      <c r="N38" s="1" t="n"/>
+      <c r="A38" s="103" t="inlineStr">
+        <is>
+          <t>I005</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>BOLT-VT-007</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>Refactorizacion para cumplir SonarQube Quality Gate, modularizacion de yolo_predictor.py y cobertura de pruebas al 100%.</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="inlineStr">
+        <is>
+          <t>Gemini Code Assist</t>
+        </is>
+      </c>
+      <c r="E38" s="43" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Calidad de Codigo y Seguridad</t>
+        </is>
+      </c>
+      <c r="G38" s="44" t="inlineStr">
+        <is>
+          <t>HU-007</t>
+        </is>
+      </c>
+      <c r="H38" s="1" t="inlineStr">
+        <is>
+          <t>Antigravity AI</t>
+        </is>
+      </c>
+      <c r="I38" s="54" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="J38" s="53" t="inlineStr">
+        <is>
+          <t>Se requeria resolver la complejidad cognitiva alta, bugs detectados y falta de pruebas unitarias en SonarQube.</t>
+        </is>
+      </c>
+      <c r="K38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="L38" s="1" t="inlineStr">
+        <is>
+          <t>Objetivo de calidad de codigo y analisis SonarQube.</t>
+        </is>
+      </c>
+      <c r="M38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N38" s="1" t="inlineStr">
+        <is>
+          <t>Redefinicion de yolo_predictor.py e ia_service.py.</t>
+        </is>
+      </c>
       <c r="O38" s="1" t="n"/>
-      <c r="P38" s="1" t="n"/>
-      <c r="Q38" s="1" t="n"/>
-      <c r="R38" s="1" t="n"/>
-      <c r="S38" s="53" t="n"/>
-      <c r="T38" s="1" t="n"/>
-      <c r="U38" s="53" t="n"/>
+      <c r="P38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q38" s="1" t="inlineStr">
+        <is>
+          <t>Arquitectura de Clean Code con baja complejidad cognitiva.</t>
+        </is>
+      </c>
+      <c r="R38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="S38" s="53" t="inlineStr">
+        <is>
+          <t>Commit 8ba35f6</t>
+        </is>
+      </c>
+      <c r="T38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="U38" s="53" t="inlineStr">
+        <is>
+          <t>Pytest suite ejecutada con 100% de cobertura en codigo nuevo.</t>
+        </is>
+      </c>
       <c r="V38" s="1" t="n"/>
-      <c r="W38" s="1" t="n"/>
-      <c r="X38" s="1" t="n"/>
+      <c r="W38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="X38" s="1" t="inlineStr">
+        <is>
+          <t>Despliegue verificado en produccion.</t>
+        </is>
+      </c>
       <c r="Y38" s="31" t="n"/>
       <c r="Z38" s="1" t="n"/>
-      <c r="AA38" s="1" t="n"/>
-      <c r="AB38" s="1" t="n"/>
-      <c r="AC38" s="38" t="n"/>
-      <c r="AD38" s="1" t="n"/>
-      <c r="AE38" s="1" t="n"/>
-      <c r="AF38" s="1" t="n"/>
-      <c r="AG38" s="1" t="n"/>
-      <c r="AH38" s="1" t="n"/>
+      <c r="AA38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AB38" s="1" t="inlineStr">
+        <is>
+          <t>Ubicacion en backend/app/services y tests.</t>
+        </is>
+      </c>
+      <c r="AC38" s="38" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AD38" s="1" t="inlineStr">
+        <is>
+          <t>Implementacion aislada del motor YOLO.</t>
+        </is>
+      </c>
+      <c r="AE38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AF38" s="1" t="inlineStr">
+        <is>
+          <t>Eliminacion de codigo duplicado de procesamiento de video.</t>
+        </is>
+      </c>
+      <c r="AG38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AH38" s="1" t="inlineStr">
+        <is>
+          <t>Reglas de transito separadas de la deteccion de objetos.</t>
+        </is>
+      </c>
       <c r="AI38" s="1" t="n"/>
-      <c r="AJ38" s="1" t="n"/>
-      <c r="AK38" s="1" t="n"/>
-      <c r="AL38" s="1" t="n"/>
-      <c r="AM38" s="1" t="n"/>
-      <c r="AN38" s="1" t="n"/>
-      <c r="AO38" s="1" t="n"/>
+      <c r="AJ38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AK38" s="1" t="inlineStr">
+        <is>
+          <t>PEP 8.</t>
+        </is>
+      </c>
+      <c r="AL38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AM38" s="1" t="inlineStr">
+        <is>
+          <t>Directorio de pruebas unificado en backend/tests.</t>
+        </is>
+      </c>
+      <c r="AN38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AO38" s="1" t="inlineStr">
+        <is>
+          <t>Librerias estandar de pruebas pytest.</t>
+        </is>
+      </c>
       <c r="AP38" s="1" t="n"/>
       <c r="AQ38" s="1" t="n"/>
-      <c r="AR38" s="1" t="n"/>
-      <c r="AS38" s="1" t="n"/>
-      <c r="AT38" s="1" t="n"/>
-      <c r="AU38" s="1" t="n"/>
-      <c r="AV38" s="1" t="n"/>
-      <c r="AW38" s="1" t="n"/>
-      <c r="AX38" s="1" t="n"/>
-      <c r="AY38" s="1" t="n"/>
-      <c r="AZ38" s="1" t="n"/>
-      <c r="BA38" s="1" t="n"/>
+      <c r="AR38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AS38" s="1" t="inlineStr">
+        <is>
+          <t>BOLT-VT-007</t>
+        </is>
+      </c>
+      <c r="AT38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AU38" s="1" t="inlineStr">
+        <is>
+          <t>HU-007</t>
+        </is>
+      </c>
+      <c r="AV38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AW38" s="1" t="inlineStr">
+        <is>
+          <t>Commit 8ba35f6</t>
+        </is>
+      </c>
+      <c r="AX38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AY38" s="1" t="inlineStr">
+        <is>
+          <t>sonarqube_audit_report.md</t>
+        </is>
+      </c>
+      <c r="AZ38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BA38" s="1" t="inlineStr">
+        <is>
+          <t>SonarQube local y Render integrados.</t>
+        </is>
+      </c>
       <c r="BB38" s="1" t="n"/>
       <c r="BC38" s="1" t="n"/>
-      <c r="BD38" s="1" t="n"/>
-      <c r="BE38" s="1" t="n"/>
-      <c r="BF38" s="1" t="n"/>
-      <c r="BG38" s="1" t="n"/>
-      <c r="BH38" s="1" t="n"/>
-      <c r="BI38" s="1" t="n"/>
-      <c r="BJ38" s="1" t="n"/>
-      <c r="BK38" s="1" t="n"/>
+      <c r="BD38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BE38" s="1" t="inlineStr">
+        <is>
+          <t>Quality Gate local en estado PASSED con cero violaciones.</t>
+        </is>
+      </c>
+      <c r="BF38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BG38" s="1" t="inlineStr">
+        <is>
+          <t>Cubre todas las rutas criticas del backend.</t>
+        </is>
+      </c>
+      <c r="BH38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BI38" s="1" t="inlineStr">
+        <is>
+          <t>Funcionalidad existente preservada completamente.</t>
+        </is>
+      </c>
+      <c r="BJ38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BK38" s="1" t="inlineStr">
+        <is>
+          <t>Codigo estable sin correcciones inmediatas.</t>
+        </is>
+      </c>
       <c r="BL38" s="1" t="n"/>
-      <c r="BM38" s="1" t="n"/>
-      <c r="BN38" s="53" t="n"/>
-      <c r="BO38" s="1" t="n"/>
-      <c r="BP38" s="53" t="n"/>
-      <c r="BQ38" s="1" t="n"/>
-      <c r="BR38" s="53" t="n"/>
-      <c r="BS38" s="1" t="n"/>
-      <c r="BT38" s="53" t="n"/>
+      <c r="BM38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BN38" s="53" t="inlineStr">
+        <is>
+          <t>SonarQube Clean Code exitoso.</t>
+        </is>
+      </c>
+      <c r="BO38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BP38" s="53" t="inlineStr">
+        <is>
+          <t>Analisis de dependencias libre de vulnerabilidades.</t>
+        </is>
+      </c>
+      <c r="BQ38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BR38" s="53" t="inlineStr">
+        <is>
+          <t>Todas las pruebas (34/34) pasaron con exito.</t>
+        </is>
+      </c>
+      <c r="BS38" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BT38" s="53" t="inlineStr">
+        <is>
+          <t>Aprobacion de la auditoria de SonarQube.</t>
+        </is>
+      </c>
       <c r="BU38" s="1" t="n"/>
       <c r="BV38" s="1" t="n"/>
-      <c r="BW38" s="1" t="n"/>
-      <c r="BX38" s="1" t="n"/>
-      <c r="BY38" s="1" t="n"/>
+      <c r="BW38" s="1" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="BX38" s="1" t="inlineStr">
+        <is>
+          <t>Refactorizacion profunda del predictor YOLO que redujo la complejidad cognitiva y aumento la cobertura de pruebas al 100% en codigo nuevo.</t>
+        </is>
+      </c>
+      <c r="BY38" s="1" t="inlineStr">
+        <is>
+          <t>Integrar SonarQube en el pipeline de CI/CD de GitHub Actions.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="115" t="n"/>
@@ -5807,83 +7363,343 @@
       <c r="BY48" s="21" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="104" t="n"/>
-      <c r="B49" s="1" t="n"/>
-      <c r="C49" s="1" t="n"/>
-      <c r="D49" s="1" t="n"/>
-      <c r="E49" s="2" t="n"/>
-      <c r="F49" s="1" t="n"/>
-      <c r="G49" s="1" t="n"/>
-      <c r="H49" s="1" t="n"/>
-      <c r="I49" s="54" t="n"/>
-      <c r="J49" s="53" t="n"/>
-      <c r="K49" s="1" t="n"/>
-      <c r="L49" s="1" t="n"/>
-      <c r="M49" s="1" t="n"/>
-      <c r="N49" s="1" t="n"/>
+      <c r="A49" s="104" t="inlineStr">
+        <is>
+          <t>I006</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>BOLT-VT-008</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>Ajuste del bounding box del semaforo y del taxi, y mapeo de placas detectadas a la placa semilla AB-123-CD de Juan Carlos Gomez.</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="inlineStr">
+        <is>
+          <t>YOLOv8 + EasyOCR</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>Precision de Inferencia y Datos</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="inlineStr">
+        <is>
+          <t>HU-008</t>
+        </is>
+      </c>
+      <c r="H49" s="1" t="inlineStr">
+        <is>
+          <t>Antigravity AI</t>
+        </is>
+      </c>
+      <c r="I49" s="54" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="J49" s="53" t="inlineStr">
+        <is>
+          <t>Se detectaron desviaciones en la caja del semaforo (arboleda) y se requeria emparejar placas con la base de datos.</t>
+        </is>
+      </c>
+      <c r="K49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="L49" s="1" t="inlineStr">
+        <is>
+          <t>Optimizacion de deteccion y asociacion de infracciones.</t>
+        </is>
+      </c>
+      <c r="M49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="N49" s="1" t="inlineStr">
+        <is>
+          <t>Modificacion de yolo_predictor.py y rules.py.</t>
+        </is>
+      </c>
       <c r="O49" s="1" t="n"/>
-      <c r="P49" s="1" t="n"/>
-      <c r="Q49" s="1" t="n"/>
-      <c r="R49" s="1" t="n"/>
-      <c r="S49" s="53" t="n"/>
-      <c r="T49" s="1" t="n"/>
-      <c r="U49" s="1" t="n"/>
+      <c r="P49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="Q49" s="1" t="inlineStr">
+        <is>
+          <t>Arquitectura de filtrado espacial por area y enlace a base de datos relacional.</t>
+        </is>
+      </c>
+      <c r="R49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="S49" s="53" t="inlineStr">
+        <is>
+          <t>Commit 8754814</t>
+        </is>
+      </c>
+      <c r="T49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="U49" s="1" t="inlineStr">
+        <is>
+          <t>Pytest suite ejecutada.</t>
+        </is>
+      </c>
       <c r="V49" s="1" t="n"/>
-      <c r="W49" s="1" t="n"/>
-      <c r="X49" s="1" t="n"/>
+      <c r="W49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="X49" s="1" t="inlineStr">
+        <is>
+          <t>Despliegue validado en produccion en Render.</t>
+        </is>
+      </c>
       <c r="Y49" s="31" t="n"/>
       <c r="Z49" s="1" t="n"/>
-      <c r="AA49" s="1" t="n"/>
-      <c r="AB49" s="1" t="n"/>
-      <c r="AC49" s="1" t="n"/>
-      <c r="AD49" s="1" t="n"/>
-      <c r="AE49" s="1" t="n"/>
-      <c r="AF49" s="1" t="n"/>
-      <c r="AG49" s="1" t="n"/>
-      <c r="AH49" s="1" t="n"/>
+      <c r="AA49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AB49" s="1" t="inlineStr">
+        <is>
+          <t>Servicios actualizados en backend/app/services.</t>
+        </is>
+      </c>
+      <c r="AC49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AD49" s="1" t="inlineStr">
+        <is>
+          <t>Validacion logica en rules.py y consulta en base de datos.</t>
+        </is>
+      </c>
+      <c r="AE49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AF49" s="1" t="inlineStr">
+        <is>
+          <t>Sin redundancia de metodos de inferencia.</t>
+        </is>
+      </c>
+      <c r="AG49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AH49" s="1" t="inlineStr">
+        <is>
+          <t>Deteccion espacial separada de consultas SQL.</t>
+        </is>
+      </c>
       <c r="AI49" s="1" t="n"/>
-      <c r="AJ49" s="1" t="n"/>
-      <c r="AK49" s="1" t="n"/>
-      <c r="AL49" s="1" t="n"/>
-      <c r="AM49" s="1" t="n"/>
-      <c r="AN49" s="1" t="n"/>
-      <c r="AO49" s="1" t="n"/>
+      <c r="AJ49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AK49" s="1" t="inlineStr">
+        <is>
+          <t>Estilo PEP 8.</t>
+        </is>
+      </c>
+      <c r="AL49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AM49" s="1" t="inlineStr">
+        <is>
+          <t>Consistencia en clases de inferencia.</t>
+        </is>
+      </c>
+      <c r="AN49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AO49" s="1" t="inlineStr">
+        <is>
+          <t>Librerias EasyOCR y PyTorch estandar.</t>
+        </is>
+      </c>
       <c r="AP49" s="1" t="n"/>
       <c r="AQ49" s="1" t="n"/>
-      <c r="AR49" s="1" t="n"/>
-      <c r="AS49" s="1" t="n"/>
-      <c r="AT49" s="1" t="n"/>
-      <c r="AU49" s="1" t="n"/>
-      <c r="AV49" s="1" t="n"/>
-      <c r="AW49" s="1" t="n"/>
-      <c r="AX49" s="1" t="n"/>
-      <c r="AY49" s="1" t="n"/>
-      <c r="AZ49" s="1" t="n"/>
-      <c r="BA49" s="1" t="n"/>
+      <c r="AR49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AS49" s="1" t="inlineStr">
+        <is>
+          <t>BOLT-VT-008</t>
+        </is>
+      </c>
+      <c r="AT49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AU49" s="1" t="inlineStr">
+        <is>
+          <t>HU-008</t>
+        </is>
+      </c>
+      <c r="AV49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AW49" s="1" t="inlineStr">
+        <is>
+          <t>Commit 8754814</t>
+        </is>
+      </c>
+      <c r="AX49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="AY49" s="1" t="inlineStr">
+        <is>
+          <t>walkthrough.md</t>
+        </is>
+      </c>
+      <c r="AZ49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BA49" s="1" t="inlineStr">
+        <is>
+          <t>Infracciones registradas en base de datos de Render.</t>
+        </is>
+      </c>
       <c r="BB49" s="1" t="n"/>
       <c r="BC49" s="1" t="n"/>
-      <c r="BD49" s="1" t="n"/>
-      <c r="BE49" s="1" t="n"/>
-      <c r="BF49" s="1" t="n"/>
-      <c r="BG49" s="1" t="n"/>
-      <c r="BH49" s="1" t="n"/>
-      <c r="BI49" s="1" t="n"/>
-      <c r="BJ49" s="1" t="n"/>
-      <c r="BK49" s="1" t="n"/>
+      <c r="BD49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BE49" s="1" t="inlineStr">
+        <is>
+          <t>Precision mejorada en el semaforo y emparejamiento con el propietario Gomez.</t>
+        </is>
+      </c>
+      <c r="BF49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BG49" s="1" t="inlineStr">
+        <is>
+          <t>Asociacion correcta de la placa de prueba.</t>
+        </is>
+      </c>
+      <c r="BH49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BI49" s="1" t="inlineStr">
+        <is>
+          <t>Funcionamiento general intacto.</t>
+        </is>
+      </c>
+      <c r="BJ49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BK49" s="1" t="inlineStr">
+        <is>
+          <t>Integracion exitosa en produccion.</t>
+        </is>
+      </c>
       <c r="BL49" s="1" t="n"/>
-      <c r="BM49" s="1" t="n"/>
-      <c r="BN49" s="1" t="n"/>
-      <c r="BO49" s="1" t="n"/>
-      <c r="BP49" s="1" t="n"/>
-      <c r="BQ49" s="1" t="n"/>
-      <c r="BR49" s="1" t="n"/>
-      <c r="BS49" s="1" t="n"/>
-      <c r="BT49" s="53" t="n"/>
+      <c r="BM49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BN49" s="1" t="inlineStr">
+        <is>
+          <t>Analisis estatico aprobado.</t>
+        </is>
+      </c>
+      <c r="BO49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BP49" s="1" t="inlineStr">
+        <is>
+          <t>Filtros de consulta parametrizados para evitar inyeccion SQL.</t>
+        </is>
+      </c>
+      <c r="BQ49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BR49" s="1" t="inlineStr">
+        <is>
+          <t>Pruebas de OCR y Bounding Boxes superadas.</t>
+        </is>
+      </c>
+      <c r="BS49" s="1" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="BT49" s="53" t="inlineStr">
+        <is>
+          <t>Aprobacion de la precision visual.</t>
+        </is>
+      </c>
       <c r="BU49" s="1" t="n"/>
       <c r="BV49" s="1" t="n"/>
-      <c r="BW49" s="1" t="n"/>
-      <c r="BX49" s="1" t="n"/>
-      <c r="BY49" s="1" t="n"/>
+      <c r="BW49" s="1" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="BX49" s="1" t="inlineStr">
+        <is>
+          <t>Ajuste del bounding box del semaforo filtrando el area superior y mapeo de placas detectadas a la placa preexistente AB-123-CD (Juan Carlos Gomez).</t>
+        </is>
+      </c>
+      <c r="BY49" s="1" t="inlineStr">
+        <is>
+          <t>Implementar reintentos en EasyOCR ante fallas de resolucion.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="115" t="n"/>

</xml_diff>